<commit_message>
chore: atualiza CONTAS-A-RECEBER.xlsx via automação (Gmail)
</commit_message>
<xml_diff>
--- a/planilhas/CONTAS-A-RECEBER.xlsx
+++ b/planilhas/CONTAS-A-RECEBER.xlsx
@@ -40,7 +40,7 @@
     </r>
   </si>
   <si>
-    <t>Relatório exportado em sexta-feira, 24 de julho de 2026 por LUZ DIVINA - FROTA 2</t>
+    <t>Relatório exportado em sábado, 25 de julho de 2026 por LUZ DIVINA - FROTA 2</t>
   </si>
   <si>
     <t>Número do Documento</t>
@@ -519,7 +519,7 @@
         <v>28</v>
       </c>
       <c r="N6" s="9">
-        <v>-53</v>
+        <v>-54</v>
       </c>
       <c r="O6" s="6" t="s">
         <v>29</v>
@@ -528,7 +528,7 @@
         <v>28</v>
       </c>
       <c r="Q6" s="9">
-        <v>-53</v>
+        <v>-54</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>29</v>
@@ -578,7 +578,7 @@
         <v>28</v>
       </c>
       <c r="N7" s="9">
-        <v>-46</v>
+        <v>-47</v>
       </c>
       <c r="O7" s="6" t="s">
         <v>29</v>
@@ -587,7 +587,7 @@
         <v>28</v>
       </c>
       <c r="Q7" s="9">
-        <v>-46</v>
+        <v>-47</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>29</v>
@@ -637,7 +637,7 @@
         <v>28</v>
       </c>
       <c r="N8" s="9">
-        <v>-39</v>
+        <v>-40</v>
       </c>
       <c r="O8" s="6" t="s">
         <v>29</v>
@@ -646,7 +646,7 @@
         <v>28</v>
       </c>
       <c r="Q8" s="9">
-        <v>-39</v>
+        <v>-40</v>
       </c>
       <c r="R8" s="6" t="s">
         <v>29</v>
@@ -696,7 +696,7 @@
         <v>28</v>
       </c>
       <c r="N9" s="9">
-        <v>-32</v>
+        <v>-33</v>
       </c>
       <c r="O9" s="6" t="s">
         <v>29</v>
@@ -705,7 +705,7 @@
         <v>28</v>
       </c>
       <c r="Q9" s="9">
-        <v>-32</v>
+        <v>-33</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
@@ -755,7 +755,7 @@
         <v>28</v>
       </c>
       <c r="N10" s="9">
-        <v>-32</v>
+        <v>-33</v>
       </c>
       <c r="O10" s="6" t="s">
         <v>29</v>
@@ -764,7 +764,7 @@
         <v>28</v>
       </c>
       <c r="Q10" s="9">
-        <v>-32</v>
+        <v>-33</v>
       </c>
       <c r="R10" s="6" t="s">
         <v>29</v>
@@ -814,7 +814,7 @@
         <v>28</v>
       </c>
       <c r="N11" s="9">
-        <v>-25</v>
+        <v>-26</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>38</v>
@@ -823,7 +823,7 @@
         <v>28</v>
       </c>
       <c r="Q11" s="9">
-        <v>-25</v>
+        <v>-26</v>
       </c>
       <c r="R11" s="6" t="s">
         <v>38</v>
@@ -873,7 +873,7 @@
         <v>28</v>
       </c>
       <c r="N12" s="9">
-        <v>-25</v>
+        <v>-26</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>38</v>
@@ -882,7 +882,7 @@
         <v>28</v>
       </c>
       <c r="Q12" s="9">
-        <v>-25</v>
+        <v>-26</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>38</v>
@@ -932,7 +932,7 @@
         <v>28</v>
       </c>
       <c r="N13" s="9">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>38</v>
@@ -941,7 +941,7 @@
         <v>28</v>
       </c>
       <c r="Q13" s="9">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>38</v>
@@ -991,7 +991,7 @@
         <v>28</v>
       </c>
       <c r="N14" s="9">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>38</v>
@@ -1000,7 +1000,7 @@
         <v>28</v>
       </c>
       <c r="Q14" s="9">
-        <v>-67</v>
+        <v>-68</v>
       </c>
       <c r="R14" s="6" t="s">
         <v>29</v>
@@ -1050,7 +1050,7 @@
         <v>28</v>
       </c>
       <c r="N15" s="9">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="O15" s="6" t="s">
         <v>38</v>
@@ -1059,7 +1059,7 @@
         <v>28</v>
       </c>
       <c r="Q15" s="9">
-        <v>-60</v>
+        <v>-61</v>
       </c>
       <c r="R15" s="6" t="s">
         <v>29</v>
@@ -1109,7 +1109,7 @@
         <v>28</v>
       </c>
       <c r="N16" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>38</v>
@@ -1118,7 +1118,7 @@
         <v>28</v>
       </c>
       <c r="Q16" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="R16" s="6" t="s">
         <v>38</v>
@@ -1168,7 +1168,7 @@
         <v>28</v>
       </c>
       <c r="N17" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="O17" s="6" t="s">
         <v>38</v>
@@ -1177,7 +1177,7 @@
         <v>28</v>
       </c>
       <c r="Q17" s="9">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="R17" s="6" t="s">
         <v>38</v>
@@ -1227,7 +1227,7 @@
         <v>28</v>
       </c>
       <c r="N18" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>38</v>
@@ -1236,7 +1236,7 @@
         <v>28</v>
       </c>
       <c r="Q18" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="R18" s="6" t="s">
         <v>38</v>
@@ -1286,7 +1286,7 @@
         <v>28</v>
       </c>
       <c r="N19" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="O19" s="6" t="s">
         <v>38</v>
@@ -1295,7 +1295,7 @@
         <v>28</v>
       </c>
       <c r="Q19" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="R19" s="6" t="s">
         <v>38</v>
@@ -1345,7 +1345,7 @@
         <v>28</v>
       </c>
       <c r="N20" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>38</v>
@@ -1354,7 +1354,7 @@
         <v>28</v>
       </c>
       <c r="Q20" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="R20" s="6" t="s">
         <v>38</v>
@@ -1404,7 +1404,7 @@
         <v>28</v>
       </c>
       <c r="N21" s="9">
-        <v>-15</v>
+        <v>-16</v>
       </c>
       <c r="O21" s="6" t="s">
         <v>38</v>
@@ -1413,7 +1413,7 @@
         <v>28</v>
       </c>
       <c r="Q21" s="9">
-        <v>-25</v>
+        <v>-26</v>
       </c>
       <c r="R21" s="6" t="s">
         <v>38</v>
@@ -1463,7 +1463,7 @@
         <v>28</v>
       </c>
       <c r="N22" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>38</v>
@@ -1472,7 +1472,7 @@
         <v>28</v>
       </c>
       <c r="Q22" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R22" s="6" t="s">
         <v>38</v>
@@ -1522,7 +1522,7 @@
         <v>28</v>
       </c>
       <c r="N23" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O23" s="6" t="s">
         <v>38</v>
@@ -1531,7 +1531,7 @@
         <v>50</v>
       </c>
       <c r="Q23" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R23" s="6" t="s">
         <v>24</v>
@@ -1581,7 +1581,7 @@
         <v>28</v>
       </c>
       <c r="N24" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>38</v>
@@ -1590,7 +1590,7 @@
         <v>28</v>
       </c>
       <c r="Q24" s="9">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="R24" s="6" t="s">
         <v>38</v>
@@ -1640,7 +1640,7 @@
         <v>28</v>
       </c>
       <c r="N25" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O25" s="6" t="s">
         <v>38</v>
@@ -1649,7 +1649,7 @@
         <v>28</v>
       </c>
       <c r="Q25" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R25" s="6" t="s">
         <v>38</v>
@@ -1699,7 +1699,7 @@
         <v>28</v>
       </c>
       <c r="N26" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>38</v>
@@ -1708,7 +1708,7 @@
         <v>28</v>
       </c>
       <c r="Q26" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R26" s="6" t="s">
         <v>38</v>
@@ -1758,7 +1758,7 @@
         <v>28</v>
       </c>
       <c r="N27" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O27" s="6" t="s">
         <v>38</v>
@@ -1767,7 +1767,7 @@
         <v>28</v>
       </c>
       <c r="Q27" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R27" s="6" t="s">
         <v>38</v>
@@ -1817,7 +1817,7 @@
         <v>28</v>
       </c>
       <c r="N28" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>38</v>
@@ -1826,7 +1826,7 @@
         <v>28</v>
       </c>
       <c r="Q28" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R28" s="6" t="s">
         <v>38</v>
@@ -1876,7 +1876,7 @@
         <v>28</v>
       </c>
       <c r="N29" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O29" s="6" t="s">
         <v>38</v>
@@ -1885,7 +1885,7 @@
         <v>28</v>
       </c>
       <c r="Q29" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R29" s="6" t="s">
         <v>38</v>
@@ -1935,7 +1935,7 @@
         <v>28</v>
       </c>
       <c r="N30" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>38</v>
@@ -1944,7 +1944,7 @@
         <v>28</v>
       </c>
       <c r="Q30" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R30" s="6" t="s">
         <v>38</v>
@@ -1994,7 +1994,7 @@
         <v>28</v>
       </c>
       <c r="N31" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O31" s="6" t="s">
         <v>38</v>
@@ -2003,7 +2003,7 @@
         <v>28</v>
       </c>
       <c r="Q31" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R31" s="6" t="s">
         <v>38</v>
@@ -2053,7 +2053,7 @@
         <v>28</v>
       </c>
       <c r="N32" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>38</v>
@@ -2062,7 +2062,7 @@
         <v>28</v>
       </c>
       <c r="Q32" s="9">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="R32" s="6" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
chore: atualiza CONTAS-A-RECEBER.xlsx via upload no Dashboard
</commit_message>
<xml_diff>
--- a/planilhas/CONTAS-A-RECEBER.xlsx
+++ b/planilhas/CONTAS-A-RECEBER.xlsx
@@ -9,14 +9,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Relatório!$A$5:$S$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$85</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -36,7 +36,7 @@
         <color rgb="FF808080"/>
         <sz val="11"/>
       </rPr>
-      <t>Data Final: 13/07/2026</t>
+      <t>Data Final: 02/08/2026</t>
     </r>
   </si>
   <si>
@@ -236,6 +236,219 @@
   </si>
   <si>
     <t>ANNY KATARINA ACIOLE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11831</t>
+  </si>
+  <si>
+    <t>OLIZIEL DA SILVA CARDOSO</t>
+  </si>
+  <si>
+    <t>FA-11943</t>
+  </si>
+  <si>
+    <t>RICARDO ARAUJO DE MIRANDA</t>
+  </si>
+  <si>
+    <t>FA-11899</t>
+  </si>
+  <si>
+    <t>FA-11837</t>
+  </si>
+  <si>
+    <t>ANDERSON QUEIROZ PINHEIRO</t>
+  </si>
+  <si>
+    <t>FA-11849</t>
+  </si>
+  <si>
+    <t>MAICON LOPES SILVA</t>
+  </si>
+  <si>
+    <t>AZ EMPREENDIMENTOS</t>
+  </si>
+  <si>
+    <t>FA-11881</t>
+  </si>
+  <si>
+    <t>FA-11911</t>
+  </si>
+  <si>
+    <t>FA-11915</t>
+  </si>
+  <si>
+    <t>FA-11987</t>
+  </si>
+  <si>
+    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
+  </si>
+  <si>
+    <t>FA-11968</t>
+  </si>
+  <si>
+    <t>ADRIANO SANTOS DE CARVALHO</t>
+  </si>
+  <si>
+    <t>FA-11945</t>
+  </si>
+  <si>
+    <t>FA-11969</t>
+  </si>
+  <si>
+    <t>FA-11856</t>
+  </si>
+  <si>
+    <t>ANDRE CAVALCANTI DA FE</t>
+  </si>
+  <si>
+    <t>FA-11629</t>
+  </si>
+  <si>
+    <t>DANILO DE ALMEIDA TORRES</t>
+  </si>
+  <si>
+    <t>FA-11961</t>
+  </si>
+  <si>
+    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
+  </si>
+  <si>
+    <t>FA-11988</t>
+  </si>
+  <si>
+    <t>ELSON VIEIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11838</t>
+  </si>
+  <si>
+    <t>FA-11839</t>
+  </si>
+  <si>
+    <t>FA-11907</t>
+  </si>
+  <si>
+    <t>FA-11949</t>
+  </si>
+  <si>
+    <t>FA-11840</t>
+  </si>
+  <si>
+    <t>FA-11989</t>
+  </si>
+  <si>
+    <t>JACKSON CASSIANO VERISSIMO</t>
+  </si>
+  <si>
+    <t>LUZ DIVINA LTDA</t>
+  </si>
+  <si>
+    <t>FA-11906</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11886</t>
+  </si>
+  <si>
+    <t>FA-11905</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11740</t>
+  </si>
+  <si>
+    <t>FA-11855</t>
+  </si>
+  <si>
+    <t>FA-12007</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11973</t>
+  </si>
+  <si>
+    <t>JOZILDO TARQUINO DE BRITO</t>
+  </si>
+  <si>
+    <t>FA-11971</t>
+  </si>
+  <si>
+    <t>FA-11993</t>
+  </si>
+  <si>
+    <t>FA-11974</t>
+  </si>
+  <si>
+    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
+  </si>
+  <si>
+    <t>FA-11947</t>
+  </si>
+  <si>
+    <t>FA-11994</t>
+  </si>
+  <si>
+    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11920</t>
+  </si>
+  <si>
+    <t>MATHEUS MATIAS CORTEZ TRIGUEIRO</t>
+  </si>
+  <si>
+    <t>FA-11857</t>
+  </si>
+  <si>
+    <t>FA-11665</t>
+  </si>
+  <si>
+    <t>LUCA ZOLI</t>
+  </si>
+  <si>
+    <t>FA-11972</t>
+  </si>
+  <si>
+    <t>FA-11992</t>
+  </si>
+  <si>
+    <t>FA-11932</t>
+  </si>
+  <si>
+    <t>WESCLY JEAN DE MEDEIROS</t>
+  </si>
+  <si>
+    <t>FA-11962</t>
+  </si>
+  <si>
+    <t>FA-11865</t>
+  </si>
+  <si>
+    <t>FA-11950</t>
+  </si>
+  <si>
+    <t>FA-11653</t>
+  </si>
+  <si>
+    <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
+  </si>
+  <si>
+    <t>PÚBLICO</t>
+  </si>
+  <si>
+    <t>FA-11991</t>
+  </si>
+  <si>
+    <t>FA-11641</t>
+  </si>
+  <si>
+    <t>TANIELLE GLAUCIANA SOUZA DA SILVA</t>
   </si>
 </sst>
 </file>
@@ -378,12 +591,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName=""/>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S85"/>
   <sheetFormatPr defaultRowHeight="23" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1" style="1"/>
     <col min="2" max="2" width="39" customWidth="1" style="1"/>
-    <col min="3" max="3" width="31" customWidth="1" style="1"/>
+    <col min="3" max="3" width="35" customWidth="1" style="1"/>
     <col min="4" max="4" width="14" customWidth="1" style="1"/>
     <col min="5" max="5" width="38" customWidth="1" style="1"/>
     <col min="6" max="6" width="16" customWidth="1" style="1"/>
@@ -2071,28 +2284,3096 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" ht="23" customHeight="1">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="12">
-        <f>SUM(L6:L32)</f>
-      </c>
-      <c r="M33" s="10"/>
-      <c r="N33" s="13"/>
-      <c r="O33" s="10"/>
-      <c r="P33" s="10"/>
-      <c r="Q33" s="13"/>
-      <c r="R33" s="10"/>
-      <c r="S33" s="10"/>
+    <row r="33">
+      <c r="A33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="7">
+        <v>46209</v>
+      </c>
+      <c r="J33" s="7">
+        <v>46220</v>
+      </c>
+      <c r="K33" s="7">
+        <v>46209</v>
+      </c>
+      <c r="L33" s="8">
+        <v>600</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N33" s="9">
+        <v>-11</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q33" s="9">
+        <v>-22</v>
+      </c>
+      <c r="R33" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S33" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I34" s="7">
+        <v>46216</v>
+      </c>
+      <c r="J34" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K34" s="7">
+        <v>46216</v>
+      </c>
+      <c r="L34" s="8">
+        <v>40</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N34" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q34" s="9">
+        <v>-15</v>
+      </c>
+      <c r="R34" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S34" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G35" s="7">
+        <v>46190</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I35" s="7">
+        <v>46174</v>
+      </c>
+      <c r="J35" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K35" s="7">
+        <v>46239</v>
+      </c>
+      <c r="L35" s="8">
+        <v>50</v>
+      </c>
+      <c r="M35" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N35" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P35" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q35" s="9">
+        <v>8</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="S35" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G36" s="7">
+        <v>46153</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I36" s="7">
+        <v>46143</v>
+      </c>
+      <c r="J36" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K36" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L36" s="8">
+        <v>50</v>
+      </c>
+      <c r="M36" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N36" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q36" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S36" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I37" s="7">
+        <v>46209</v>
+      </c>
+      <c r="J37" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K37" s="7">
+        <v>46209</v>
+      </c>
+      <c r="L37" s="8">
+        <v>60</v>
+      </c>
+      <c r="M37" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N37" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O37" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q37" s="9">
+        <v>-22</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S37" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I38" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J38" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K38" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L38" s="8">
+        <v>76.01</v>
+      </c>
+      <c r="M38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N38" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O38" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q38" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R38" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S38" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I39" s="7">
+        <v>46188</v>
+      </c>
+      <c r="J39" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K39" s="7">
+        <v>46188</v>
+      </c>
+      <c r="L39" s="8">
+        <v>96.66</v>
+      </c>
+      <c r="M39" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N39" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O39" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P39" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q39" s="9">
+        <v>-43</v>
+      </c>
+      <c r="R39" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="S39" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I40" s="7">
+        <v>46209</v>
+      </c>
+      <c r="J40" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K40" s="7">
+        <v>46209</v>
+      </c>
+      <c r="L40" s="8">
+        <v>200</v>
+      </c>
+      <c r="M40" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N40" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O40" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P40" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q40" s="9">
+        <v>-22</v>
+      </c>
+      <c r="R40" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S40" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I41" s="7">
+        <v>46209</v>
+      </c>
+      <c r="J41" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K41" s="7">
+        <v>46209</v>
+      </c>
+      <c r="L41" s="8">
+        <v>330</v>
+      </c>
+      <c r="M41" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N41" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O41" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P41" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q41" s="9">
+        <v>-22</v>
+      </c>
+      <c r="R41" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S41" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G42" s="7">
+        <v>46203</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I42" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J42" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K42" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L42" s="8">
+        <v>630</v>
+      </c>
+      <c r="M42" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N42" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O42" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P42" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q42" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R42" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S42" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I43" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J43" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K43" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L43" s="8">
+        <v>630</v>
+      </c>
+      <c r="M43" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N43" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P43" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q43" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R43" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S43" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G44" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I44" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J44" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K44" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L44" s="8">
+        <v>630</v>
+      </c>
+      <c r="M44" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N44" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O44" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P44" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q44" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R44" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S44" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G45" s="7">
+        <v>46212</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I45" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J45" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K45" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L45" s="8">
+        <v>630</v>
+      </c>
+      <c r="M45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N45" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O45" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q45" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R45" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S45" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G46" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I46" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J46" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K46" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L46" s="8">
+        <v>650</v>
+      </c>
+      <c r="M46" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N46" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O46" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P46" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q46" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R46" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S46" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="7">
+        <v>46188</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I47" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J47" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K47" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L47" s="8">
+        <v>650</v>
+      </c>
+      <c r="M47" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N47" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O47" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P47" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q47" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R47" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S47" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G48" s="7">
+        <v>46153</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I48" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J48" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K48" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L48" s="8">
+        <v>650</v>
+      </c>
+      <c r="M48" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N48" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O48" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P48" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q48" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R48" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S48" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G49" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I49" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J49" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K49" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L49" s="8">
+        <v>680</v>
+      </c>
+      <c r="M49" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N49" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O49" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P49" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q49" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R49" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S49" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I50" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J50" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K50" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L50" s="8">
+        <v>680</v>
+      </c>
+      <c r="M50" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N50" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O50" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P50" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q50" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R50" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S50" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G51" s="7">
+        <v>46182</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I51" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J51" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K51" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L51" s="8">
+        <v>680</v>
+      </c>
+      <c r="M51" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N51" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O51" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P51" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q51" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R51" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S51" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G52" s="7">
+        <v>46182</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I52" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J52" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K52" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L52" s="8">
+        <v>680</v>
+      </c>
+      <c r="M52" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N52" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O52" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P52" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q52" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R52" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S52" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G53" s="7">
+        <v>46203</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I53" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J53" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K53" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L53" s="8">
+        <v>700</v>
+      </c>
+      <c r="M53" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N53" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O53" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P53" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q53" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R53" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S53" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I54" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J54" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K54" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L54" s="8">
+        <v>800</v>
+      </c>
+      <c r="M54" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N54" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O54" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P54" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q54" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R54" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S54" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G55" s="7">
+        <v>46182</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I55" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J55" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K55" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L55" s="8">
+        <v>800</v>
+      </c>
+      <c r="M55" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N55" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O55" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P55" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q55" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R55" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S55" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I56" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J56" s="7">
+        <v>46223</v>
+      </c>
+      <c r="K56" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L56" s="8">
+        <v>1200</v>
+      </c>
+      <c r="M56" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N56" s="9">
+        <v>-8</v>
+      </c>
+      <c r="O56" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P56" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q56" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R56" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S56" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I57" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J57" s="7">
+        <v>46224</v>
+      </c>
+      <c r="K57" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L57" s="8">
+        <v>3.91</v>
+      </c>
+      <c r="M57" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N57" s="9">
+        <v>-7</v>
+      </c>
+      <c r="O57" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P57" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q57" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R57" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S57" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I58" s="7">
+        <v>46216</v>
+      </c>
+      <c r="J58" s="7">
+        <v>46224</v>
+      </c>
+      <c r="K58" s="7">
+        <v>46216</v>
+      </c>
+      <c r="L58" s="8">
+        <v>56.19</v>
+      </c>
+      <c r="M58" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N58" s="9">
+        <v>-7</v>
+      </c>
+      <c r="O58" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P58" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q58" s="9">
+        <v>-15</v>
+      </c>
+      <c r="R58" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S58" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I59" s="7">
+        <v>46223</v>
+      </c>
+      <c r="J59" s="7">
+        <v>46224</v>
+      </c>
+      <c r="K59" s="7">
+        <v>46223</v>
+      </c>
+      <c r="L59" s="8">
+        <v>71</v>
+      </c>
+      <c r="M59" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N59" s="9">
+        <v>-7</v>
+      </c>
+      <c r="O59" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P59" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q59" s="9">
+        <v>-8</v>
+      </c>
+      <c r="R59" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S59" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G60" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I60" s="7">
+        <v>46216</v>
+      </c>
+      <c r="J60" s="7">
+        <v>46224</v>
+      </c>
+      <c r="K60" s="7">
+        <v>46216</v>
+      </c>
+      <c r="L60" s="8">
+        <v>360.95</v>
+      </c>
+      <c r="M60" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N60" s="9">
+        <v>-7</v>
+      </c>
+      <c r="O60" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P60" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q60" s="9">
+        <v>-15</v>
+      </c>
+      <c r="R60" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S60" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I61" s="7">
+        <v>46216</v>
+      </c>
+      <c r="J61" s="7">
+        <v>46224</v>
+      </c>
+      <c r="K61" s="7">
+        <v>46216</v>
+      </c>
+      <c r="L61" s="8">
+        <v>550</v>
+      </c>
+      <c r="M61" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N61" s="9">
+        <v>-7</v>
+      </c>
+      <c r="O61" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P61" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q61" s="9">
+        <v>-15</v>
+      </c>
+      <c r="R61" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S61" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G62" s="7">
+        <v>46190</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I62" s="7">
+        <v>46174</v>
+      </c>
+      <c r="J62" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K62" s="7">
+        <v>46246</v>
+      </c>
+      <c r="L62" s="8">
+        <v>50</v>
+      </c>
+      <c r="M62" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N62" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O62" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P62" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q62" s="9">
+        <v>15</v>
+      </c>
+      <c r="R62" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="S62" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G63" s="7">
+        <v>46153</v>
+      </c>
+      <c r="H63" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I63" s="7">
+        <v>46143</v>
+      </c>
+      <c r="J63" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K63" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L63" s="8">
+        <v>50</v>
+      </c>
+      <c r="M63" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N63" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O63" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P63" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q63" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R63" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S63" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I64" s="7">
+        <v>46188</v>
+      </c>
+      <c r="J64" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K64" s="7">
+        <v>46188</v>
+      </c>
+      <c r="L64" s="8">
+        <v>116.66</v>
+      </c>
+      <c r="M64" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N64" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O64" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P64" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q64" s="9">
+        <v>-43</v>
+      </c>
+      <c r="R64" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="S64" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G65" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I65" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J65" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K65" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L65" s="8">
+        <v>600</v>
+      </c>
+      <c r="M65" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N65" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O65" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P65" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q65" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R65" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S65" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G66" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I66" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J66" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K66" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L66" s="8">
+        <v>600</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N66" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O66" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P66" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q66" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R66" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S66" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G67" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I67" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J67" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K67" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L67" s="8">
+        <v>630</v>
+      </c>
+      <c r="M67" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N67" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O67" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P67" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q67" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R67" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S67" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G68" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I68" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J68" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K68" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L68" s="8">
+        <v>630</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N68" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O68" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P68" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q68" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R68" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S68" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G69" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I69" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J69" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K69" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L69" s="8">
+        <v>630</v>
+      </c>
+      <c r="M69" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N69" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O69" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P69" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q69" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R69" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S69" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G70" s="7">
+        <v>46212</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I70" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J70" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K70" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L70" s="8">
+        <v>630</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N70" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O70" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P70" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q70" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R70" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S70" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G71" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I71" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J71" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K71" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L71" s="8">
+        <v>630</v>
+      </c>
+      <c r="M71" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N71" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O71" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P71" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q71" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R71" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S71" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G72" s="7">
+        <v>46210</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I72" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J72" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K72" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L72" s="8">
+        <v>650</v>
+      </c>
+      <c r="M72" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N72" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O72" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P72" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q72" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R72" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S72" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G73" s="7">
+        <v>46188</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I73" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J73" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K73" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L73" s="8">
+        <v>650</v>
+      </c>
+      <c r="M73" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N73" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O73" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P73" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q73" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R73" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S73" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G74" s="7">
+        <v>46160</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I74" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J74" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K74" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L74" s="8">
+        <v>650</v>
+      </c>
+      <c r="M74" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N74" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P74" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q74" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R74" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S74" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G75" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I75" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J75" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K75" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L75" s="8">
+        <v>650</v>
+      </c>
+      <c r="M75" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N75" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O75" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P75" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q75" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R75" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S75" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G76" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I76" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J76" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K76" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L76" s="8">
+        <v>680</v>
+      </c>
+      <c r="M76" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N76" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O76" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P76" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q76" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R76" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S76" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G77" s="7">
+        <v>46212</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I77" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J77" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K77" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L77" s="8">
+        <v>680</v>
+      </c>
+      <c r="M77" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N77" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O77" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P77" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q77" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R77" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S77" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G78" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I78" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J78" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K78" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L78" s="8">
+        <v>680</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N78" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O78" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P78" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q78" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R78" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S78" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G79" s="7">
+        <v>46188</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I79" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J79" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K79" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L79" s="8">
+        <v>700</v>
+      </c>
+      <c r="M79" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N79" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O79" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P79" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q79" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R79" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S79" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G80" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I80" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J80" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K80" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L80" s="8">
+        <v>800</v>
+      </c>
+      <c r="M80" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N80" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O80" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P80" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q80" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R80" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S80" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G81" s="7">
+        <v>46160</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I81" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J81" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K81" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L81" s="8">
+        <v>1200</v>
+      </c>
+      <c r="M81" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N81" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O81" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P81" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q81" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R81" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S81" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G82" s="7">
+        <v>46225</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I82" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J82" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K82" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L82" s="8">
+        <v>1200</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N82" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O82" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P82" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q82" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R82" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S82" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G83" s="7">
+        <v>46160</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I83" s="7">
+        <v>46230</v>
+      </c>
+      <c r="J83" s="7">
+        <v>46230</v>
+      </c>
+      <c r="K83" s="7">
+        <v>46230</v>
+      </c>
+      <c r="L83" s="8">
+        <v>1200</v>
+      </c>
+      <c r="M83" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N83" s="9">
+        <v>-1</v>
+      </c>
+      <c r="O83" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P83" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q83" s="9">
+        <v>-1</v>
+      </c>
+      <c r="R83" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S83" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G84" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I84" s="7">
+        <v>45930</v>
+      </c>
+      <c r="J84" s="7">
+        <v>46233</v>
+      </c>
+      <c r="K84" s="7">
+        <v>46233</v>
+      </c>
+      <c r="L84" s="8">
+        <v>185.5</v>
+      </c>
+      <c r="M84" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N84" s="9">
+        <v>2</v>
+      </c>
+      <c r="O84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="P84" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q84" s="9">
+        <v>2</v>
+      </c>
+      <c r="R84" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="S84" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="85" ht="23" customHeight="1">
+      <c r="A85" s="10"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="10"/>
+      <c r="E85" s="10"/>
+      <c r="F85" s="10"/>
+      <c r="G85" s="11"/>
+      <c r="H85" s="10"/>
+      <c r="I85" s="11"/>
+      <c r="J85" s="11"/>
+      <c r="K85" s="11"/>
+      <c r="L85" s="12">
+        <f>SUM(L6:L84)</f>
+      </c>
+      <c r="M85" s="10"/>
+      <c r="N85" s="13"/>
+      <c r="O85" s="10"/>
+      <c r="P85" s="10"/>
+      <c r="Q85" s="13"/>
+      <c r="R85" s="10"/>
+      <c r="S85" s="10"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:S5"/>

</xml_diff>